<commit_message>
chore: sincronizar estado atualizado das cotacoes
</commit_message>
<xml_diff>
--- a/cotacoes_pesquisa_mercado.xlsx
+++ b/cotacoes_pesquisa_mercado.xlsx
@@ -709,42 +709,52 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Pendente de Cotação</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
+          <t>Cotado e Homologado</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>70.69</v>
+      </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Não Localizado</t>
+          <t>Loja SRVGÁS</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>33.200.056/0001-49</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Dupla Pesquisa Externa (CNPJ loja)</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Pendente de Cotação</t>
+          <t>Regulador de pressão 2kg Aliança 506/01</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Pesquisa comercial realizada, mas nenhum e-commerce com CNPJ comprovado atendeu à especificação nesta rodada.</t>
+          <t>O valor foi extraído diretamente da página do produto (Regulador de pressão 2kg Aliança 506/01). Os demais valores listados no JSON original (R$ 35,75, R$ 121,27, R$ 124,91 e R$ 104,40) referem-se a produtos relacionados (outros modelos de reguladores) exibidos na seção de recomendações da página, sendo descartados por não corresponderem ao item solicitado.</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>27/10/2026 às 10:30:48</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
+          <t>27/10/2026 às 10:35:40</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>https://loja.srvgas.com.br/produto/regulador-de-pressao-2kg-alianca-506-01/</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>prints_cotacoes\lote_004_REGULADOR_DE_PRESSÃO_2KG_H_5.png</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">

</xml_diff>

<commit_message>
feat: iniciar servidor web automaticamente em background (porta 5000)
</commit_message>
<xml_diff>
--- a/cotacoes_pesquisa_mercado.xlsx
+++ b/cotacoes_pesquisa_mercado.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -545,12 +545,12 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Preço unitário extraído conforme anúncio de venda avulsa de vasilhame de 20 litros (garrafão plástico vazio). Não há menção a pacotes ou lotes, tratando-se de unidade única.</t>
+          <t>Preço unitário extraído diretamente da página do produto. Não há menção a pacotes ou lotes, tratando-se de venda individual por unidade (vasilhame).</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>27/10/2026 às 10:30:12</t>
+          <t>27/10/2026 às 10:37:55</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -585,16 +585,16 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>5.95</v>
+        <v>2.2</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Ultrafarma</t>
+          <t>Kalunga</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>02.543.945/0006-90</t>
+          <t>43.283.811/0001-50</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -604,22 +604,22 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Água Mineral Sem Gás 500ml - Embalagem Renovável</t>
+          <t>Água Mineral sem gás, 500ml, Pack com 12 unidades, Crystal FD 12 UN</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>O valor unitário foi extraído do preço de venda padrão ('Por') indicado na página. Desconsiderou-se o valor promocional de Pix (R$ 5,77) para fins de pesquisa de mercado, seguindo a diretriz de utilizar o preço de venda geral ofertado ao público.</t>
+          <t>O valor total do pack com 12 unidades é R$ 26,40. O valor unitário foi obtido pela divisão R$ 26,40 / 12 = R$ 2,20.</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>27/10/2026 às 10:30:31</t>
+          <t>27/10/2026 às 10:38:18</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>https://www.ultrafarma.com.br/agua-mineral-sem-gas-500ml-embalagem-renovavel</t>
+          <t>https://www.kalunga.com.br/prod/agua-mineral-sem-gas-500ml-pack-com-12-unidades-crystal-fd-12-un/996944</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -649,41 +649,41 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>1.41</v>
+        <v>4.49</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Cristal Select</t>
+          <t>Pague Menos</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>33.200.056/0001-49</t>
+          <t>06.626.253/0001-51</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Base Oficial de Redes Elétricas</t>
+          <t>Dupla Pesquisa Externa (CNPJ paguemenos)</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Água Mineral Cristal Select 500ml Com Gás Pacote com 12 Unidades</t>
+          <t>Água Mineral Acqualia Com Gás 500ml</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>O preço de R$ 16,90 refere-se à compra única de um pacote com 12 unidades. O valor unitário foi obtido pela divisão do preço do pacote (R$ 16,90) pela quantidade de itens (12), resultando em R$ 1,4083, arredondado para R$ 1,41 conforme informado no anúncio original.</t>
+          <t>O valor foi extraído do destaque principal da página (R$ 4,49 por unidade de 500ml). Os demais valores detectados (como R$ 12,49) referem-se a variações de packs ou pacotes não especificados, prevalecendo o valor unitário nominal identificado para a embalagem de 500ml.</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>27/10/2026 às 10:35:01</t>
+          <t>27/10/2026 às 10:38:45</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>https://loja.cristalselect.com.br/products/agua-mineral-cristal-select-500ml-com-gas-fardo-com-12-unidades</t>
+          <t>https://www.paguemenos.com.br/agua-mineral-acqualia-com-gas-500ml/p</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -713,110 +713,46 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>70.69</v>
+        <v>61.9</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Loja SRVGÁS</t>
+          <t>Aliança Metalúrgica</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>33.200.056/0001-49</t>
+          <t>52.012.582/0001-20</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Dupla Pesquisa Externa (CNPJ loja)</t>
+          <t>Dupla Pesquisa Externa (CNPJ paravoce)</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Regulador de pressão 2kg Aliança 506/01</t>
+          <t>Regulador de Gás Doméstico 506/01 Aliança</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>O valor foi extraído diretamente da página do produto (Regulador de pressão 2kg Aliança 506/01). Os demais valores listados no JSON original (R$ 35,75, R$ 121,27, R$ 124,91 e R$ 104,40) referem-se a produtos relacionados (outros modelos de reguladores) exibidos na seção de recomendações da página, sendo descartados por não corresponderem ao item solicitado.</t>
+          <t>O valor de R$61,90 foi extraído diretamente do anúncio do produto. O valor R$6,19 refere-se a uma parcela de 10x, o valor R$67,90 refere-se a produtos relacionados (505/01) e o status do item é 'ESGOTADO', fator que deve ser considerado na análise de viabilidade de contratação conforme Lei 14.133/2021.</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>27/10/2026 às 10:35:40</t>
+          <t>27/10/2026 às 10:38:57</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>https://loja.srvgas.com.br/produto/regulador-de-pressao-2kg-alianca-506-01/</t>
+          <t>https://paravoce.aliancametalurgica.com.br/produtos/regulador-de-gas-domestico-506-01-alianca/</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
           <t>prints_cotacoes\lote_004_REGULADOR_DE_PRESSÃO_2KG_H_5.png</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>MANGUEIRA MULTIUSO 3/8X4MM TRANÇADA</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>UNID</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Cotado e Homologado</t>
-        </is>
-      </c>
-      <c r="F6" t="n">
-        <v>4.53</v>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Elite Gás</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>10.838.714/0001-27</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Dupla Pesquisa Externa (CNPJ elitegas)</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>Mangueira 3/8 X 4mm 11k 50 Metros Trançada Multiuso</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>O preço de R$ 226,65 refere-se a um rolo de 50 metros do produto. O valor unitário foi obtido pela divisão do valor total pela metragem (226,65 / 50 = 4,533). Considerou-se o preço à vista (PIX) para maior precisão na estimativa de mercado.</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>27/10/2026 às 10:31:02</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>https://www.elitegas.com.br/produtos/mangueira-3-8-x-4mm-11k-50-metros-trancada-multiuso/</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>prints_cotacoes\lote_005_MANGUEIRA_MULTIUSO_3_8X4MM_T.png</t>
         </is>
       </c>
     </row>

</xml_diff>